<commit_message>
simple wght log skill dropped
</commit_message>
<xml_diff>
--- a/inst/simple_summ_plot/quarterly_summary.xlsx
+++ b/inst/simple_summ_plot/quarterly_summary.xlsx
@@ -425,20 +425,20 @@
         <v>39994</v>
       </c>
       <c r="D2" t="n">
-        <v>61.81</v>
+        <v>61.842</v>
       </c>
       <c r="E2" t="n">
-        <v>0.001</v>
+        <v>-0.002</v>
       </c>
       <c r="F2"/>
       <c r="G2" t="n">
-        <v>61.81</v>
+        <v>61.895</v>
       </c>
       <c r="H2" t="n">
-        <v>61.797</v>
+        <v>61.842</v>
       </c>
       <c r="I2" t="n">
-        <v>0.013</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="3">
@@ -452,22 +452,22 @@
         <v>40086</v>
       </c>
       <c r="D3" t="n">
-        <v>61.874</v>
+        <v>61.735</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.064</v>
+        <v>-0.107</v>
       </c>
       <c r="G3" t="n">
-        <v>61.874</v>
+        <v>61.84</v>
       </c>
       <c r="H3" t="n">
-        <v>61.81</v>
+        <v>61.735</v>
       </c>
       <c r="I3" t="n">
-        <v>0.063</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="4">
@@ -481,22 +481,22 @@
         <v>40178</v>
       </c>
       <c r="D4" t="n">
-        <v>62.007</v>
+        <v>61.945</v>
       </c>
       <c r="E4" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F4" t="n">
-        <v>0.133</v>
+        <v>0.21</v>
       </c>
       <c r="G4" t="n">
-        <v>62.007</v>
+        <v>61.945</v>
       </c>
       <c r="H4" t="n">
-        <v>61.874</v>
+        <v>61.735</v>
       </c>
       <c r="I4" t="n">
-        <v>0.132</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="5">
@@ -510,22 +510,22 @@
         <v>40268</v>
       </c>
       <c r="D5" t="n">
-        <v>62.622</v>
+        <v>62.838</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="F5" t="n">
-        <v>0.615</v>
+        <v>0.893</v>
       </c>
       <c r="G5" t="n">
-        <v>62.622</v>
+        <v>62.838</v>
       </c>
       <c r="H5" t="n">
-        <v>62.009</v>
+        <v>61.95</v>
       </c>
       <c r="I5" t="n">
-        <v>0.613</v>
+        <v>0.888</v>
       </c>
     </row>
     <row r="6">
@@ -539,22 +539,22 @@
         <v>40359</v>
       </c>
       <c r="D6" t="n">
-        <v>64.644</v>
+        <v>64.632</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.042</v>
+        <v>-0.06</v>
       </c>
       <c r="F6" t="n">
-        <v>2.022</v>
+        <v>1.794</v>
       </c>
       <c r="G6" t="n">
-        <v>65.255</v>
+        <v>65.315</v>
       </c>
       <c r="H6" t="n">
-        <v>62.642</v>
+        <v>62.858</v>
       </c>
       <c r="I6" t="n">
-        <v>2.612</v>
+        <v>2.458</v>
       </c>
     </row>
     <row r="7">
@@ -568,22 +568,22 @@
         <v>40451</v>
       </c>
       <c r="D7" t="n">
-        <v>64.059</v>
+        <v>64.242</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.021</v>
+        <v>0.004</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.585</v>
+        <v>-0.39</v>
       </c>
       <c r="G7" t="n">
-        <v>64.603</v>
+        <v>64.572</v>
       </c>
       <c r="H7" t="n">
-        <v>63.904</v>
+        <v>63.933</v>
       </c>
       <c r="I7" t="n">
-        <v>0.699</v>
+        <v>0.639</v>
       </c>
     </row>
     <row r="8">
@@ -597,22 +597,22 @@
         <v>40543</v>
       </c>
       <c r="D8" t="n">
-        <v>64.213</v>
+        <v>65.001</v>
       </c>
       <c r="E8" t="n">
-        <v>0.02</v>
+        <v>0.012</v>
       </c>
       <c r="F8" t="n">
-        <v>0.155</v>
+        <v>0.759</v>
       </c>
       <c r="G8" t="n">
-        <v>64.213</v>
+        <v>65.001</v>
       </c>
       <c r="H8" t="n">
-        <v>63.633</v>
+        <v>64.247</v>
       </c>
       <c r="I8" t="n">
-        <v>0.581</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="9">
@@ -626,22 +626,22 @@
         <v>40633</v>
       </c>
       <c r="D9" t="n">
-        <v>66.661</v>
+        <v>66.333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.029</v>
+        <v>0.018</v>
       </c>
       <c r="F9" t="n">
-        <v>2.448</v>
+        <v>1.332</v>
       </c>
       <c r="G9" t="n">
-        <v>66.661</v>
+        <v>66.333</v>
       </c>
       <c r="H9" t="n">
-        <v>64.234</v>
+        <v>65.013</v>
       </c>
       <c r="I9" t="n">
-        <v>2.427</v>
+        <v>1.321</v>
       </c>
     </row>
     <row r="10">
@@ -655,22 +655,22 @@
         <v>40724</v>
       </c>
       <c r="D10" t="n">
-        <v>68.362</v>
+        <v>68.05</v>
       </c>
       <c r="E10" t="n">
-        <v>0.003</v>
+        <v>0.015</v>
       </c>
       <c r="F10" t="n">
-        <v>1.701</v>
+        <v>1.717</v>
       </c>
       <c r="G10" t="n">
-        <v>68.362</v>
+        <v>68.05</v>
       </c>
       <c r="H10" t="n">
-        <v>66.69</v>
+        <v>66.351</v>
       </c>
       <c r="I10" t="n">
-        <v>1.672</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="11">
@@ -684,22 +684,22 @@
         <v>40816</v>
       </c>
       <c r="D11" t="n">
-        <v>66.135</v>
+        <v>66.542</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.057</v>
+        <v>-0.063</v>
       </c>
       <c r="F11" t="n">
-        <v>-2.227</v>
+        <v>-1.508</v>
       </c>
       <c r="G11" t="n">
-        <v>68.372</v>
+        <v>68.287</v>
       </c>
       <c r="H11" t="n">
-        <v>66.135</v>
+        <v>66.542</v>
       </c>
       <c r="I11" t="n">
-        <v>2.237</v>
+        <v>1.745</v>
       </c>
     </row>
     <row r="12">
@@ -713,22 +713,22 @@
         <v>40908</v>
       </c>
       <c r="D12" t="n">
-        <v>61.069</v>
+        <v>63.107</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.028</v>
+        <v>-0.002</v>
       </c>
       <c r="F12" t="n">
-        <v>-5.066</v>
+        <v>-3.435</v>
       </c>
       <c r="G12" t="n">
-        <v>66.077</v>
+        <v>66.479</v>
       </c>
       <c r="H12" t="n">
-        <v>61.069</v>
+        <v>63.107</v>
       </c>
       <c r="I12" t="n">
-        <v>5.009</v>
+        <v>3.372</v>
       </c>
     </row>
     <row r="13">
@@ -742,22 +742,22 @@
         <v>40999</v>
       </c>
       <c r="D13" t="n">
-        <v>62.294</v>
+        <v>63.905</v>
       </c>
       <c r="E13" t="n">
-        <v>0.038</v>
+        <v>0.014</v>
       </c>
       <c r="F13" t="n">
-        <v>1.226</v>
+        <v>0.798</v>
       </c>
       <c r="G13" t="n">
-        <v>62.294</v>
+        <v>63.905</v>
       </c>
       <c r="H13" t="n">
-        <v>60.744</v>
+        <v>63.103</v>
       </c>
       <c r="I13" t="n">
-        <v>1.551</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="14">
@@ -771,22 +771,22 @@
         <v>41090</v>
       </c>
       <c r="D14" t="n">
-        <v>64.839</v>
+        <v>64.712</v>
       </c>
       <c r="E14" t="n">
-        <v>0.006</v>
+        <v>0.009</v>
       </c>
       <c r="F14" t="n">
-        <v>2.545</v>
+        <v>0.807</v>
       </c>
       <c r="G14" t="n">
-        <v>64.839</v>
+        <v>64.712</v>
       </c>
       <c r="H14" t="n">
-        <v>62.332</v>
+        <v>63.919</v>
       </c>
       <c r="I14" t="n">
-        <v>2.507</v>
+        <v>0.793</v>
       </c>
     </row>
     <row r="15">
@@ -800,22 +800,22 @@
         <v>41182</v>
       </c>
       <c r="D15" t="n">
-        <v>65.731</v>
+        <v>66.362</v>
       </c>
       <c r="E15" t="n">
-        <v>0.026</v>
+        <v>0.025</v>
       </c>
       <c r="F15" t="n">
-        <v>0.892</v>
+        <v>1.65</v>
       </c>
       <c r="G15" t="n">
-        <v>65.731</v>
+        <v>66.362</v>
       </c>
       <c r="H15" t="n">
-        <v>64.845</v>
+        <v>64.721</v>
       </c>
       <c r="I15" t="n">
-        <v>0.887</v>
+        <v>1.641</v>
       </c>
     </row>
     <row r="16">
@@ -829,22 +829,22 @@
         <v>41274</v>
       </c>
       <c r="D16" t="n">
-        <v>68.998</v>
+        <v>68.872</v>
       </c>
       <c r="E16" t="n">
-        <v>0.039</v>
+        <v>0.027</v>
       </c>
       <c r="F16" t="n">
-        <v>3.267</v>
+        <v>2.51</v>
       </c>
       <c r="G16" t="n">
-        <v>68.998</v>
+        <v>68.872</v>
       </c>
       <c r="H16" t="n">
-        <v>65.757</v>
+        <v>66.387</v>
       </c>
       <c r="I16" t="n">
-        <v>3.241</v>
+        <v>2.485</v>
       </c>
     </row>
     <row r="17">
@@ -858,22 +858,22 @@
         <v>41364</v>
       </c>
       <c r="D17" t="n">
-        <v>71.79</v>
+        <v>70.95</v>
       </c>
       <c r="E17" t="n">
         <v>0.017</v>
       </c>
       <c r="F17" t="n">
-        <v>2.792</v>
+        <v>2.078</v>
       </c>
       <c r="G17" t="n">
-        <v>71.79</v>
+        <v>70.95</v>
       </c>
       <c r="H17" t="n">
-        <v>69.037</v>
+        <v>68.899</v>
       </c>
       <c r="I17" t="n">
-        <v>2.753</v>
+        <v>2.051</v>
       </c>
     </row>
     <row r="18">
@@ -887,22 +887,22 @@
         <v>41455</v>
       </c>
       <c r="D18" t="n">
-        <v>71.005</v>
+        <v>71.337</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.04</v>
+        <v>-0.032</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.785</v>
+        <v>0.387</v>
       </c>
       <c r="G18" t="n">
-        <v>72.093</v>
+        <v>71.55</v>
       </c>
       <c r="H18" t="n">
-        <v>71.005</v>
+        <v>70.966</v>
       </c>
       <c r="I18" t="n">
-        <v>1.088</v>
+        <v>0.583</v>
       </c>
     </row>
     <row r="19">
@@ -916,22 +916,22 @@
         <v>41547</v>
       </c>
       <c r="D19" t="n">
-        <v>69.979</v>
+        <v>69.851</v>
       </c>
       <c r="E19" t="n">
-        <v>0.028</v>
+        <v>0.025</v>
       </c>
       <c r="F19" t="n">
-        <v>-1.026</v>
+        <v>-1.487</v>
       </c>
       <c r="G19" t="n">
-        <v>70.964</v>
+        <v>71.303</v>
       </c>
       <c r="H19" t="n">
-        <v>68.864</v>
+        <v>68.646</v>
       </c>
       <c r="I19" t="n">
-        <v>2.101</v>
+        <v>2.658</v>
       </c>
     </row>
     <row r="20">
@@ -945,22 +945,22 @@
         <v>41639</v>
       </c>
       <c r="D20" t="n">
-        <v>71.668</v>
+        <v>71.918</v>
       </c>
       <c r="E20" t="n">
-        <v>0.006</v>
+        <v>0.011</v>
       </c>
       <c r="F20" t="n">
-        <v>1.689</v>
+        <v>2.068</v>
       </c>
       <c r="G20" t="n">
-        <v>71.668</v>
+        <v>71.918</v>
       </c>
       <c r="H20" t="n">
-        <v>70.004</v>
+        <v>69.876</v>
       </c>
       <c r="I20" t="n">
-        <v>1.663</v>
+        <v>2.042</v>
       </c>
     </row>
     <row r="21">
@@ -974,22 +974,22 @@
         <v>41729</v>
       </c>
       <c r="D21" t="n">
-        <v>72.083</v>
+        <v>72.152</v>
       </c>
       <c r="E21" t="n">
-        <v>0.004</v>
+        <v>-0.002</v>
       </c>
       <c r="F21" t="n">
-        <v>0.416</v>
+        <v>0.233</v>
       </c>
       <c r="G21" t="n">
-        <v>72.083</v>
+        <v>72.188</v>
       </c>
       <c r="H21" t="n">
-        <v>71.673</v>
+        <v>71.929</v>
       </c>
       <c r="I21" t="n">
-        <v>0.41</v>
+        <v>0.258</v>
       </c>
     </row>
     <row r="22">
@@ -1003,22 +1003,22 @@
         <v>41820</v>
       </c>
       <c r="D22" t="n">
-        <v>72.364</v>
+        <v>72.137</v>
       </c>
       <c r="E22" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F22" t="n">
-        <v>0.28</v>
+        <v>-0.015</v>
       </c>
       <c r="G22" t="n">
-        <v>72.364</v>
+        <v>72.15</v>
       </c>
       <c r="H22" t="n">
-        <v>72.087</v>
+        <v>72.103</v>
       </c>
       <c r="I22" t="n">
-        <v>0.277</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="23">
@@ -1032,22 +1032,22 @@
         <v>41912</v>
       </c>
       <c r="D23" t="n">
-        <v>72.638</v>
+        <v>72.431</v>
       </c>
       <c r="E23" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="F23" t="n">
-        <v>0.274</v>
+        <v>0.295</v>
       </c>
       <c r="G23" t="n">
-        <v>72.638</v>
+        <v>72.431</v>
       </c>
       <c r="H23" t="n">
-        <v>72.366</v>
+        <v>72.138</v>
       </c>
       <c r="I23" t="n">
-        <v>0.272</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="24">
@@ -1061,22 +1061,22 @@
         <v>42004</v>
       </c>
       <c r="D24" t="n">
-        <v>73.04</v>
+        <v>72.985</v>
       </c>
       <c r="E24" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="F24" t="n">
-        <v>0.402</v>
+        <v>0.554</v>
       </c>
       <c r="G24" t="n">
-        <v>73.04</v>
+        <v>72.985</v>
       </c>
       <c r="H24" t="n">
-        <v>72.642</v>
+        <v>72.436</v>
       </c>
       <c r="I24" t="n">
-        <v>0.398</v>
+        <v>0.549</v>
       </c>
     </row>
     <row r="25">
@@ -1090,22 +1090,22 @@
         <v>42094</v>
       </c>
       <c r="D25" t="n">
-        <v>73.667</v>
+        <v>73.725</v>
       </c>
       <c r="E25" t="n">
-        <v>0.008</v>
+        <v>0.009</v>
       </c>
       <c r="F25" t="n">
-        <v>0.627</v>
+        <v>0.74</v>
       </c>
       <c r="G25" t="n">
-        <v>73.667</v>
+        <v>73.725</v>
       </c>
       <c r="H25" t="n">
-        <v>73.045</v>
+        <v>72.992</v>
       </c>
       <c r="I25" t="n">
-        <v>0.621</v>
+        <v>0.733</v>
       </c>
     </row>
     <row r="26">
@@ -1119,22 +1119,22 @@
         <v>42185</v>
       </c>
       <c r="D26" t="n">
-        <v>74.516</v>
+        <v>74.62</v>
       </c>
       <c r="E26" t="n">
         <v>0.01</v>
       </c>
       <c r="F26" t="n">
-        <v>0.85</v>
+        <v>0.895</v>
       </c>
       <c r="G26" t="n">
-        <v>74.516</v>
+        <v>74.62</v>
       </c>
       <c r="H26" t="n">
-        <v>73.675</v>
+        <v>73.734</v>
       </c>
       <c r="I26" t="n">
-        <v>0.841</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="27">
@@ -1148,22 +1148,22 @@
         <v>42277</v>
       </c>
       <c r="D27" t="n">
-        <v>75.525</v>
+        <v>75.621</v>
       </c>
       <c r="E27" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="F27" t="n">
-        <v>1.008</v>
+        <v>1.001</v>
       </c>
       <c r="G27" t="n">
-        <v>75.525</v>
+        <v>75.621</v>
       </c>
       <c r="H27" t="n">
-        <v>74.527</v>
+        <v>74.63</v>
       </c>
       <c r="I27" t="n">
-        <v>0.998</v>
+        <v>0.991</v>
       </c>
     </row>
     <row r="28">
@@ -1177,22 +1177,22 @@
         <v>42369</v>
       </c>
       <c r="D28" t="n">
-        <v>76.611</v>
+        <v>76.665</v>
       </c>
       <c r="E28" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="F28" t="n">
-        <v>1.086</v>
+        <v>1.044</v>
       </c>
       <c r="G28" t="n">
-        <v>76.611</v>
+        <v>76.665</v>
       </c>
       <c r="H28" t="n">
-        <v>75.536</v>
+        <v>75.633</v>
       </c>
       <c r="I28" t="n">
-        <v>1.075</v>
+        <v>1.033</v>
       </c>
     </row>
     <row r="29">
@@ -1206,22 +1206,22 @@
         <v>42460</v>
       </c>
       <c r="D29" t="n">
-        <v>77.691</v>
+        <v>77.685</v>
       </c>
       <c r="E29" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="F29" t="n">
-        <v>1.08</v>
+        <v>1.02</v>
       </c>
       <c r="G29" t="n">
-        <v>77.691</v>
+        <v>77.685</v>
       </c>
       <c r="H29" t="n">
-        <v>76.623</v>
+        <v>76.677</v>
       </c>
       <c r="I29" t="n">
-        <v>1.068</v>
+        <v>1.009</v>
       </c>
     </row>
     <row r="30">
@@ -1235,22 +1235,22 @@
         <v>42551</v>
       </c>
       <c r="D30" t="n">
-        <v>78.706</v>
+        <v>78.638</v>
       </c>
       <c r="E30" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
       <c r="F30" t="n">
-        <v>1.015</v>
+        <v>0.953</v>
       </c>
       <c r="G30" t="n">
-        <v>78.706</v>
+        <v>78.638</v>
       </c>
       <c r="H30" t="n">
-        <v>77.703</v>
+        <v>77.696</v>
       </c>
       <c r="I30" t="n">
-        <v>1.003</v>
+        <v>0.942</v>
       </c>
     </row>
     <row r="31">
@@ -1264,22 +1264,22 @@
         <v>42643</v>
       </c>
       <c r="D31" t="n">
-        <v>79.593</v>
+        <v>79.477</v>
       </c>
       <c r="E31" t="n">
-        <v>0.009</v>
+        <v>0.008</v>
       </c>
       <c r="F31" t="n">
-        <v>0.888</v>
+        <v>0.839</v>
       </c>
       <c r="G31" t="n">
-        <v>79.593</v>
+        <v>79.477</v>
       </c>
       <c r="H31" t="n">
-        <v>78.716</v>
+        <v>78.648</v>
       </c>
       <c r="I31" t="n">
-        <v>0.877</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="32">
@@ -1293,22 +1293,22 @@
         <v>42735</v>
       </c>
       <c r="D32" t="n">
-        <v>80.27</v>
+        <v>80.136</v>
       </c>
       <c r="E32" t="n">
         <v>0.006</v>
       </c>
       <c r="F32" t="n">
-        <v>0.677</v>
+        <v>0.659</v>
       </c>
       <c r="G32" t="n">
-        <v>80.27</v>
+        <v>80.136</v>
       </c>
       <c r="H32" t="n">
-        <v>79.602</v>
+        <v>79.486</v>
       </c>
       <c r="I32" t="n">
-        <v>0.668</v>
+        <v>0.651</v>
       </c>
     </row>
     <row r="33">
@@ -1322,22 +1322,22 @@
         <v>42825</v>
       </c>
       <c r="D33" t="n">
-        <v>80.658</v>
+        <v>80.552</v>
       </c>
       <c r="E33" t="n">
         <v>0.003</v>
       </c>
       <c r="F33" t="n">
-        <v>0.388</v>
+        <v>0.416</v>
       </c>
       <c r="G33" t="n">
-        <v>80.658</v>
+        <v>80.552</v>
       </c>
       <c r="H33" t="n">
-        <v>80.276</v>
+        <v>80.142</v>
       </c>
       <c r="I33" t="n">
-        <v>0.382</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="34">
@@ -1351,22 +1351,22 @@
         <v>42916</v>
       </c>
       <c r="D34" t="n">
-        <v>80.705</v>
+        <v>80.689</v>
       </c>
       <c r="E34" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0.047</v>
+        <v>0.137</v>
       </c>
       <c r="G34" t="n">
-        <v>80.732</v>
+        <v>80.69</v>
       </c>
       <c r="H34" t="n">
-        <v>80.66</v>
+        <v>80.555</v>
       </c>
       <c r="I34" t="n">
-        <v>0.072</v>
+        <v>0.134</v>
       </c>
     </row>
     <row r="35">
@@ -1380,22 +1380,22 @@
         <v>43008</v>
       </c>
       <c r="D35" t="n">
-        <v>80.901</v>
+        <v>80.679</v>
       </c>
       <c r="E35" t="n">
-        <v>0.02</v>
+        <v>0.011</v>
       </c>
       <c r="F35" t="n">
-        <v>0.196</v>
+        <v>-0.01</v>
       </c>
       <c r="G35" t="n">
-        <v>80.901</v>
+        <v>80.689</v>
       </c>
       <c r="H35" t="n">
-        <v>80.551</v>
+        <v>80.582</v>
       </c>
       <c r="I35" t="n">
-        <v>0.349</v>
+        <v>0.107</v>
       </c>
     </row>
     <row r="36">
@@ -1409,22 +1409,22 @@
         <v>43100</v>
       </c>
       <c r="D36" t="n">
-        <v>83.408</v>
+        <v>83.165</v>
       </c>
       <c r="E36" t="n">
-        <v>0.02</v>
+        <v>0.026</v>
       </c>
       <c r="F36" t="n">
-        <v>2.508</v>
+        <v>2.486</v>
       </c>
       <c r="G36" t="n">
-        <v>83.408</v>
+        <v>83.165</v>
       </c>
       <c r="H36" t="n">
-        <v>80.921</v>
+        <v>80.69</v>
       </c>
       <c r="I36" t="n">
-        <v>2.487</v>
+        <v>2.475</v>
       </c>
     </row>
     <row r="37">
@@ -1438,22 +1438,22 @@
         <v>43190</v>
       </c>
       <c r="D37" t="n">
-        <v>82.11</v>
+        <v>82.362</v>
       </c>
       <c r="E37" t="n">
-        <v>-0.063</v>
+        <v>-0.06</v>
       </c>
       <c r="F37" t="n">
-        <v>-1.298</v>
+        <v>-0.803</v>
       </c>
       <c r="G37" t="n">
-        <v>83.761</v>
+        <v>83.745</v>
       </c>
       <c r="H37" t="n">
-        <v>82.11</v>
+        <v>82.362</v>
       </c>
       <c r="I37" t="n">
-        <v>1.651</v>
+        <v>1.383</v>
       </c>
     </row>
     <row r="38">
@@ -1467,22 +1467,22 @@
         <v>43281</v>
       </c>
       <c r="D38" t="n">
-        <v>73.373</v>
+        <v>73.552</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.036</v>
+        <v>-0.005</v>
       </c>
       <c r="F38" t="n">
-        <v>-8.738</v>
+        <v>-8.81</v>
       </c>
       <c r="G38" t="n">
-        <v>82.047</v>
+        <v>82.301</v>
       </c>
       <c r="H38" t="n">
-        <v>73.373</v>
+        <v>73.552</v>
       </c>
       <c r="I38" t="n">
-        <v>8.674</v>
+        <v>8.749</v>
       </c>
     </row>
     <row r="39">
@@ -1496,22 +1496,22 @@
         <v>43373</v>
       </c>
       <c r="D39" t="n">
-        <v>73.302</v>
+        <v>72.516</v>
       </c>
       <c r="E39" t="n">
-        <v>0.01</v>
+        <v>0.016</v>
       </c>
       <c r="F39" t="n">
-        <v>-0.071</v>
+        <v>-1.036</v>
       </c>
       <c r="G39" t="n">
-        <v>73.338</v>
+        <v>73.548</v>
       </c>
       <c r="H39" t="n">
-        <v>72.965</v>
+        <v>72.352</v>
       </c>
       <c r="I39" t="n">
-        <v>0.373</v>
+        <v>1.197</v>
       </c>
     </row>
     <row r="40">
@@ -1525,22 +1525,22 @@
         <v>43465</v>
       </c>
       <c r="D40" t="n">
-        <v>75.465</v>
+        <v>75.84</v>
       </c>
       <c r="E40" t="n">
-        <v>0.041</v>
+        <v>0.046</v>
       </c>
       <c r="F40" t="n">
-        <v>2.163</v>
+        <v>3.324</v>
       </c>
       <c r="G40" t="n">
-        <v>75.465</v>
+        <v>75.84</v>
       </c>
       <c r="H40" t="n">
-        <v>73.312</v>
+        <v>72.532</v>
       </c>
       <c r="I40" t="n">
-        <v>2.153</v>
+        <v>3.309</v>
       </c>
     </row>
     <row r="41">
@@ -1554,22 +1554,22 @@
         <v>43555</v>
       </c>
       <c r="D41" t="n">
-        <v>79.31</v>
+        <v>78.988</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.028</v>
+        <v>0.012</v>
       </c>
       <c r="F41" t="n">
-        <v>3.845</v>
+        <v>3.148</v>
       </c>
       <c r="G41" t="n">
-        <v>79.408</v>
+        <v>78.988</v>
       </c>
       <c r="H41" t="n">
-        <v>75.506</v>
+        <v>75.886</v>
       </c>
       <c r="I41" t="n">
-        <v>3.902</v>
+        <v>3.102</v>
       </c>
     </row>
     <row r="42">
@@ -1583,22 +1583,22 @@
         <v>43646</v>
       </c>
       <c r="D42" t="n">
-        <v>80.33</v>
+        <v>80.153</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.026</v>
+        <v>0.001</v>
       </c>
       <c r="F42" t="n">
-        <v>1.02</v>
+        <v>1.164</v>
       </c>
       <c r="G42" t="n">
-        <v>80.346</v>
+        <v>80.153</v>
       </c>
       <c r="H42" t="n">
-        <v>78.489</v>
+        <v>78.717</v>
       </c>
       <c r="I42" t="n">
-        <v>1.858</v>
+        <v>1.436</v>
       </c>
     </row>
     <row r="43">
@@ -1612,22 +1612,22 @@
         <v>43738</v>
       </c>
       <c r="D43" t="n">
-        <v>75.786</v>
+        <v>75.697</v>
       </c>
       <c r="E43" t="n">
-        <v>0.018</v>
+        <v>0.028</v>
       </c>
       <c r="F43" t="n">
-        <v>-4.544</v>
+        <v>-4.455</v>
       </c>
       <c r="G43" t="n">
-        <v>80.561</v>
+        <v>80.562</v>
       </c>
       <c r="H43" t="n">
-        <v>75.755</v>
+        <v>75.643</v>
       </c>
       <c r="I43" t="n">
-        <v>4.806</v>
+        <v>4.919</v>
       </c>
     </row>
     <row r="44">
@@ -1641,22 +1641,22 @@
         <v>43830</v>
       </c>
       <c r="D44" t="n">
-        <v>79.706</v>
+        <v>79.727</v>
       </c>
       <c r="E44" t="n">
-        <v>0.127</v>
+        <v>0.151</v>
       </c>
       <c r="F44" t="n">
-        <v>3.92</v>
+        <v>4.03</v>
       </c>
       <c r="G44" t="n">
-        <v>79.706</v>
+        <v>79.727</v>
       </c>
       <c r="H44" t="n">
-        <v>75.807</v>
+        <v>75.729</v>
       </c>
       <c r="I44" t="n">
-        <v>3.9</v>
+        <v>3.998</v>
       </c>
     </row>
     <row r="45">
@@ -1670,22 +1670,22 @@
         <v>43921</v>
       </c>
       <c r="D45" t="n">
-        <v>77.268</v>
+        <v>77.367</v>
       </c>
       <c r="E45" t="n">
-        <v>0.048</v>
+        <v>0.044</v>
       </c>
       <c r="F45" t="n">
-        <v>-2.438</v>
+        <v>-2.36</v>
       </c>
       <c r="G45" t="n">
-        <v>80.77</v>
+        <v>81.026</v>
       </c>
       <c r="H45" t="n">
-        <v>75.244</v>
+        <v>75.213</v>
       </c>
       <c r="I45" t="n">
-        <v>5.525</v>
+        <v>5.813</v>
       </c>
     </row>
     <row r="46">
@@ -1699,22 +1699,22 @@
         <v>44012</v>
       </c>
       <c r="D46" t="n">
-        <v>78.979</v>
+        <v>79.053</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.03</v>
+        <v>-0.037</v>
       </c>
       <c r="F46" t="n">
-        <v>1.711</v>
+        <v>1.686</v>
       </c>
       <c r="G46" t="n">
-        <v>79.227</v>
+        <v>79.256</v>
       </c>
       <c r="H46" t="n">
-        <v>77.315</v>
+        <v>77.408</v>
       </c>
       <c r="I46" t="n">
-        <v>1.912</v>
+        <v>1.847</v>
       </c>
     </row>
     <row r="47">
@@ -1728,22 +1728,22 @@
         <v>44104</v>
       </c>
       <c r="D47" t="n">
-        <v>75.026</v>
+        <v>75.043</v>
       </c>
       <c r="E47" t="n">
-        <v>0.023</v>
+        <v>0.033</v>
       </c>
       <c r="F47" t="n">
-        <v>-3.953</v>
+        <v>-4.01</v>
       </c>
       <c r="G47" t="n">
-        <v>78.949</v>
+        <v>79.015</v>
       </c>
       <c r="H47" t="n">
-        <v>74.861</v>
+        <v>74.797</v>
       </c>
       <c r="I47" t="n">
-        <v>4.088</v>
+        <v>4.217</v>
       </c>
     </row>
     <row r="48">
@@ -1757,22 +1757,22 @@
         <v>44196</v>
       </c>
       <c r="D48" t="n">
-        <v>78.109</v>
+        <v>78.255</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.019</v>
+        <v>0.01</v>
       </c>
       <c r="F48" t="n">
-        <v>3.083</v>
+        <v>3.213</v>
       </c>
       <c r="G48" t="n">
-        <v>78.163</v>
+        <v>78.255</v>
       </c>
       <c r="H48" t="n">
-        <v>75.05</v>
+        <v>75.075</v>
       </c>
       <c r="I48" t="n">
-        <v>3.114</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="49">
@@ -1786,22 +1786,22 @@
         <v>44286</v>
       </c>
       <c r="D49" t="n">
-        <v>82.272</v>
+        <v>82.428</v>
       </c>
       <c r="E49" t="n">
-        <v>0.02</v>
+        <v>0.007</v>
       </c>
       <c r="F49" t="n">
-        <v>4.164</v>
+        <v>4.173</v>
       </c>
       <c r="G49" t="n">
-        <v>82.272</v>
+        <v>82.428</v>
       </c>
       <c r="H49" t="n">
-        <v>77.966</v>
+        <v>78.101</v>
       </c>
       <c r="I49" t="n">
-        <v>4.306</v>
+        <v>4.327</v>
       </c>
     </row>
     <row r="50">
@@ -1815,22 +1815,22 @@
         <v>44377</v>
       </c>
       <c r="D50" t="n">
-        <v>84.135</v>
+        <v>84.234</v>
       </c>
       <c r="E50" t="n">
-        <v>-0.059</v>
+        <v>-0.065</v>
       </c>
       <c r="F50" t="n">
-        <v>1.863</v>
+        <v>1.807</v>
       </c>
       <c r="G50" t="n">
-        <v>84.473</v>
+        <v>84.46</v>
       </c>
       <c r="H50" t="n">
-        <v>82.292</v>
+        <v>82.308</v>
       </c>
       <c r="I50" t="n">
-        <v>2.181</v>
+        <v>2.152</v>
       </c>
     </row>
     <row r="51">
@@ -1844,22 +1844,22 @@
         <v>44469</v>
       </c>
       <c r="D51" t="n">
-        <v>86.236</v>
+        <v>85.537</v>
       </c>
       <c r="E51" t="n">
-        <v>0.031</v>
+        <v>0.025</v>
       </c>
       <c r="F51" t="n">
-        <v>2.101</v>
+        <v>1.303</v>
       </c>
       <c r="G51" t="n">
-        <v>86.236</v>
+        <v>85.537</v>
       </c>
       <c r="H51" t="n">
-        <v>82.847</v>
+        <v>82.931</v>
       </c>
       <c r="I51" t="n">
-        <v>3.389</v>
+        <v>2.606</v>
       </c>
     </row>
     <row r="52">
@@ -1873,22 +1873,22 @@
         <v>44561</v>
       </c>
       <c r="D52" t="n">
-        <v>81.681</v>
+        <v>81.571</v>
       </c>
       <c r="E52" t="n">
-        <v>-0.01</v>
+        <v>-0.043</v>
       </c>
       <c r="F52" t="n">
-        <v>-4.555</v>
+        <v>-3.966</v>
       </c>
       <c r="G52" t="n">
-        <v>86.394</v>
+        <v>85.686</v>
       </c>
       <c r="H52" t="n">
-        <v>81.681</v>
+        <v>81.571</v>
       </c>
       <c r="I52" t="n">
-        <v>4.713</v>
+        <v>4.115</v>
       </c>
     </row>
     <row r="53">
@@ -1902,22 +1902,22 @@
         <v>44651</v>
       </c>
       <c r="D53" t="n">
-        <v>84.612</v>
+        <v>84.699</v>
       </c>
       <c r="E53" t="n">
-        <v>0.01</v>
+        <v>-0.005</v>
       </c>
       <c r="F53" t="n">
-        <v>2.931</v>
+        <v>3.128</v>
       </c>
       <c r="G53" t="n">
-        <v>84.612</v>
+        <v>84.715</v>
       </c>
       <c r="H53" t="n">
-        <v>81.671</v>
+        <v>81.411</v>
       </c>
       <c r="I53" t="n">
-        <v>2.941</v>
+        <v>3.304</v>
       </c>
     </row>
     <row r="54">
@@ -1931,22 +1931,22 @@
         <v>44742</v>
       </c>
       <c r="D54" t="n">
-        <v>83.974</v>
+        <v>83.995</v>
       </c>
       <c r="E54" t="n">
-        <v>-0.002</v>
+        <v>-0.006</v>
       </c>
       <c r="F54" t="n">
-        <v>-0.638</v>
+        <v>-0.704</v>
       </c>
       <c r="G54" t="n">
         <v>84.693</v>
       </c>
       <c r="H54" t="n">
-        <v>83.974</v>
+        <v>83.995</v>
       </c>
       <c r="I54" t="n">
-        <v>0.719</v>
+        <v>0.698</v>
       </c>
     </row>
     <row r="55">
@@ -1960,22 +1960,22 @@
         <v>44834</v>
       </c>
       <c r="D55" t="n">
-        <v>85.889</v>
+        <v>85.861</v>
       </c>
       <c r="E55" t="n">
-        <v>0.025</v>
+        <v>0.033</v>
       </c>
       <c r="F55" t="n">
-        <v>1.915</v>
+        <v>1.866</v>
       </c>
       <c r="G55" t="n">
-        <v>85.889</v>
+        <v>85.861</v>
       </c>
       <c r="H55" t="n">
-        <v>83.972</v>
+        <v>83.97</v>
       </c>
       <c r="I55" t="n">
-        <v>1.917</v>
+        <v>1.892</v>
       </c>
     </row>
     <row r="56">
@@ -1989,22 +1989,22 @@
         <v>44926</v>
       </c>
       <c r="D56" t="n">
-        <v>86.144</v>
+        <v>86.029</v>
       </c>
       <c r="E56" t="n">
-        <v>-0.003</v>
+        <v>0.004</v>
       </c>
       <c r="F56" t="n">
-        <v>0.255</v>
+        <v>0.168</v>
       </c>
       <c r="G56" t="n">
-        <v>86.367</v>
+        <v>86.502</v>
       </c>
       <c r="H56" t="n">
-        <v>85.914</v>
+        <v>85.894</v>
       </c>
       <c r="I56" t="n">
-        <v>0.453</v>
+        <v>0.607</v>
       </c>
     </row>
     <row r="57">
@@ -2018,22 +2018,22 @@
         <v>45016</v>
       </c>
       <c r="D57" t="n">
-        <v>86.129</v>
+        <v>86.254</v>
       </c>
       <c r="E57" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.014</v>
+        <v>0.225</v>
       </c>
       <c r="G57" t="n">
-        <v>86.141</v>
+        <v>86.254</v>
       </c>
       <c r="H57" t="n">
-        <v>86.076</v>
+        <v>86.033</v>
       </c>
       <c r="I57" t="n">
-        <v>0.065</v>
+        <v>0.221</v>
       </c>
     </row>
     <row r="58">
@@ -2047,22 +2047,22 @@
         <v>45107</v>
       </c>
       <c r="D58" t="n">
-        <v>86.242</v>
+        <v>86.206</v>
       </c>
       <c r="E58" t="n">
-        <v>-0.001</v>
+        <v>0.001</v>
       </c>
       <c r="F58" t="n">
-        <v>0.112</v>
+        <v>-0.047</v>
       </c>
       <c r="G58" t="n">
-        <v>86.246</v>
+        <v>86.253</v>
       </c>
       <c r="H58" t="n">
-        <v>86.131</v>
+        <v>86.203</v>
       </c>
       <c r="I58" t="n">
-        <v>0.114</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="59">
@@ -2076,22 +2076,22 @@
         <v>45199</v>
       </c>
       <c r="D59" t="n">
-        <v>86.552</v>
+        <v>86.455</v>
       </c>
       <c r="E59" t="n">
-        <v>0.009</v>
+        <v>0.003</v>
       </c>
       <c r="F59" t="n">
-        <v>0.311</v>
+        <v>0.249</v>
       </c>
       <c r="G59" t="n">
-        <v>86.552</v>
+        <v>86.455</v>
       </c>
       <c r="H59" t="n">
-        <v>86.225</v>
+        <v>86.207</v>
       </c>
       <c r="I59" t="n">
-        <v>0.327</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="60">
@@ -2105,22 +2105,22 @@
         <v>45291</v>
       </c>
       <c r="D60" t="n">
-        <v>86.144</v>
+        <v>86.058</v>
       </c>
       <c r="E60" t="n">
-        <v>0.041</v>
+        <v>0.034</v>
       </c>
       <c r="F60" t="n">
-        <v>-0.408</v>
+        <v>-0.397</v>
       </c>
       <c r="G60" t="n">
-        <v>86.722</v>
+        <v>86.495</v>
       </c>
       <c r="H60" t="n">
-        <v>85.87</v>
+        <v>85.907</v>
       </c>
       <c r="I60" t="n">
-        <v>0.852</v>
+        <v>0.588</v>
       </c>
     </row>
     <row r="61">
@@ -2134,22 +2134,22 @@
         <v>45382</v>
       </c>
       <c r="D61" t="n">
-        <v>82.008</v>
+        <v>82.121</v>
       </c>
       <c r="E61" t="n">
-        <v>-0.015</v>
+        <v>-0.006</v>
       </c>
       <c r="F61" t="n">
-        <v>-4.136</v>
+        <v>-3.937</v>
       </c>
       <c r="G61" t="n">
-        <v>86.329</v>
+        <v>86.296</v>
       </c>
       <c r="H61" t="n">
-        <v>82.008</v>
+        <v>82.121</v>
       </c>
       <c r="I61" t="n">
-        <v>4.321</v>
+        <v>4.175</v>
       </c>
     </row>
     <row r="62">
@@ -2163,22 +2163,22 @@
         <v>45473</v>
       </c>
       <c r="D62" t="n">
-        <v>80.136</v>
+        <v>80.355</v>
       </c>
       <c r="E62" t="n">
-        <v>-0.021</v>
+        <v>-0.023</v>
       </c>
       <c r="F62" t="n">
-        <v>-1.873</v>
+        <v>-1.766</v>
       </c>
       <c r="G62" t="n">
-        <v>82.149</v>
+        <v>82.116</v>
       </c>
       <c r="H62" t="n">
-        <v>80.136</v>
+        <v>80.355</v>
       </c>
       <c r="I62" t="n">
-        <v>2.013</v>
+        <v>1.761</v>
       </c>
     </row>
     <row r="63">
@@ -2192,22 +2192,22 @@
         <v>45565</v>
       </c>
       <c r="D63" t="n">
-        <v>80.987</v>
+        <v>80.871</v>
       </c>
       <c r="E63" t="n">
-        <v>0.007</v>
+        <v>0.011</v>
       </c>
       <c r="F63" t="n">
-        <v>0.851</v>
+        <v>0.515</v>
       </c>
       <c r="G63" t="n">
-        <v>80.987</v>
+        <v>80.871</v>
       </c>
       <c r="H63" t="n">
-        <v>79.998</v>
+        <v>80.015</v>
       </c>
       <c r="I63" t="n">
-        <v>0.989</v>
+        <v>0.856</v>
       </c>
     </row>
     <row r="64">
@@ -2221,22 +2221,22 @@
         <v>45657</v>
       </c>
       <c r="D64" t="n">
-        <v>81.089</v>
+        <v>81.327</v>
       </c>
       <c r="E64" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>0.102</v>
+        <v>0.456</v>
       </c>
       <c r="G64" t="n">
-        <v>81.156</v>
+        <v>81.327</v>
       </c>
       <c r="H64" t="n">
-        <v>80.994</v>
+        <v>80.882</v>
       </c>
       <c r="I64" t="n">
-        <v>0.162</v>
+        <v>0.445</v>
       </c>
     </row>
     <row r="65">
@@ -2250,22 +2250,22 @@
         <v>45747</v>
       </c>
       <c r="D65" t="n">
-        <v>80.875</v>
+        <v>81.065</v>
       </c>
       <c r="E65" t="n">
-        <v>-0.001</v>
+        <v>-0.004</v>
       </c>
       <c r="F65" t="n">
-        <v>-0.214</v>
+        <v>-0.262</v>
       </c>
       <c r="G65" t="n">
-        <v>81.086</v>
+        <v>81.326</v>
       </c>
       <c r="H65" t="n">
-        <v>80.875</v>
+        <v>81.065</v>
       </c>
       <c r="I65" t="n">
-        <v>0.211</v>
+        <v>0.261</v>
       </c>
     </row>
     <row r="66">
@@ -2279,22 +2279,22 @@
         <v>45838</v>
       </c>
       <c r="D66" t="n">
-        <v>80.919</v>
+        <v>80.747</v>
       </c>
       <c r="E66" t="n">
-        <v>0.002</v>
+        <v>-0.002</v>
       </c>
       <c r="F66" t="n">
-        <v>0.043</v>
+        <v>-0.318</v>
       </c>
       <c r="G66" t="n">
-        <v>80.919</v>
+        <v>81.061</v>
       </c>
       <c r="H66" t="n">
-        <v>80.862</v>
+        <v>80.747</v>
       </c>
       <c r="I66" t="n">
-        <v>0.057</v>
+        <v>0.313</v>
       </c>
     </row>
     <row r="67">
@@ -2308,22 +2308,22 @@
         <v>45930</v>
       </c>
       <c r="D67" t="n">
-        <v>81.18</v>
+        <v>80.811</v>
       </c>
       <c r="E67" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F67" t="n">
-        <v>0.261</v>
+        <v>0.064</v>
       </c>
       <c r="G67" t="n">
-        <v>81.18</v>
+        <v>80.811</v>
       </c>
       <c r="H67" t="n">
-        <v>80.92</v>
+        <v>80.725</v>
       </c>
       <c r="I67" t="n">
-        <v>0.26</v>
+        <v>0.086</v>
       </c>
     </row>
     <row r="68">
@@ -2337,22 +2337,22 @@
         <v>46022</v>
       </c>
       <c r="D68" t="n">
-        <v>81.588</v>
+        <v>81.185</v>
       </c>
       <c r="E68" t="n">
         <v>0.005</v>
       </c>
       <c r="F68" t="n">
-        <v>0.408</v>
+        <v>0.373</v>
       </c>
       <c r="G68" t="n">
-        <v>81.588</v>
+        <v>81.185</v>
       </c>
       <c r="H68" t="n">
-        <v>81.184</v>
+        <v>80.814</v>
       </c>
       <c r="I68" t="n">
-        <v>0.404</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="69">
@@ -2366,22 +2366,22 @@
         <v>46112</v>
       </c>
       <c r="D69" t="n">
-        <v>82.06</v>
+        <v>81.706</v>
       </c>
       <c r="E69" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="F69" t="n">
-        <v>0.472</v>
+        <v>0.522</v>
       </c>
       <c r="G69" t="n">
-        <v>82.06</v>
+        <v>81.706</v>
       </c>
       <c r="H69" t="n">
-        <v>81.593</v>
+        <v>81.19</v>
       </c>
       <c r="I69" t="n">
-        <v>0.467</v>
+        <v>0.517</v>
       </c>
     </row>
     <row r="70">
@@ -2392,25 +2392,25 @@
         <v>9</v>
       </c>
       <c r="C70" s="1" t="n">
-        <v>46146</v>
+        <v>46151</v>
       </c>
       <c r="D70" t="n">
-        <v>82.243</v>
+        <v>81.946</v>
       </c>
       <c r="E70" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="F70" t="n">
-        <v>0.183</v>
+        <v>0.24</v>
       </c>
       <c r="G70" t="n">
-        <v>82.243</v>
+        <v>81.946</v>
       </c>
       <c r="H70" t="n">
-        <v>82.065</v>
+        <v>81.712</v>
       </c>
       <c r="I70" t="n">
-        <v>0.178</v>
+        <v>0.233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>